<commit_message>
프레임워크 업데이트, Table 및 Record를 사용하는 CharacterDataProcessFeature추가, itemRecord 따로 작성, FishModule -> FishFeature 이름 수정, 데이터 필드 상단으로 이동
</commit_message>
<xml_diff>
--- a/Assets/Project/Csv/Item/1. Equipment.xlsx
+++ b/Assets/Project/Csv/Item/1. Equipment.xlsx
@@ -1,29 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4507"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ycjun\OneDrive\문서\Projects\Git\GitLab\Dairy Farm\Assets\Project\Csv\Item\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A058164B-8EBA-442E-8C53-8FB0E59CF3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="3120" windowWidth="21600" windowHeight="11295"/>
+    <workbookView xWindow="0" yWindow="870" windowWidth="9180" windowHeight="8385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="125725"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -40,14 +35,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>index</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>nameTag</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve"> description</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -85,14 +72,22 @@
   </si>
   <si>
     <t>낚시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>name</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,7 +190,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -247,7 +242,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -461,16 +456,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
@@ -480,15 +475,15 @@
     <col min="6" max="6" width="13.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>4</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -497,18 +492,18 @@
         <v>1</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -520,15 +515,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -540,15 +535,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -560,15 +555,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5">
         <v>1</v>

</xml_diff>